<commit_message>
Add short attendance section in faculty dashboard
</commit_message>
<xml_diff>
--- a/backend/src/uploads/attendance-reports/Attendance_IT301_2026-06.xlsx
+++ b/backend/src/uploads/attendance-reports/Attendance_IT301_2026-06.xlsx
@@ -136,7 +136,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>20.00%</t>
+    <t>32.00%</t>
   </si>
   <si>
     <t>0801IT221002</t>
@@ -145,7 +145,7 @@
     <t>Bob Verma</t>
   </si>
   <si>
-    <t>70.00%</t>
+    <t>76.00%</t>
   </si>
 </sst>
 </file>
@@ -169,10 +169,10 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF006100"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -189,11 +189,6 @@
         <fgColor rgb="FFFDE8E8"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF4CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -207,13 +202,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -714,49 +708,49 @@
         <v>40</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="Y2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AC2" s="2" t="s">
         <v>38</v>
@@ -765,131 +759,131 @@
         <v>38</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AG2" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AH2" s="2">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="AI2" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="AJ2" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AC3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AE3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AF3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AG3" s="4">
-        <v>7</v>
-      </c>
-      <c r="AH3" s="4">
-        <v>3</v>
-      </c>
-      <c r="AI3" s="4">
-        <v>10</v>
-      </c>
-      <c r="AJ3" s="5" t="s">
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" t="s">
+        <v>40</v>
+      </c>
+      <c r="S3" t="s">
+        <v>39</v>
+      </c>
+      <c r="T3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG3">
+        <v>19</v>
+      </c>
+      <c r="AH3">
+        <v>6</v>
+      </c>
+      <c r="AI3">
+        <v>25</v>
+      </c>
+      <c r="AJ3" s="4" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update admin contact functionality
</commit_message>
<xml_diff>
--- a/backend/src/uploads/attendance-reports/Attendance_IT301_2026-06.xlsx
+++ b/backend/src/uploads/attendance-reports/Attendance_IT301_2026-06.xlsx
@@ -136,7 +136,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>20.00%</t>
+    <t>27.27%</t>
   </si>
   <si>
     <t>0801IT221002</t>
@@ -145,7 +145,7 @@
     <t>Bob Verma</t>
   </si>
   <si>
-    <t>70.00%</t>
+    <t>72.73%</t>
   </si>
 </sst>
 </file>
@@ -714,7 +714,7 @@
         <v>40</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>38</v>
@@ -771,13 +771,13 @@
         <v>38</v>
       </c>
       <c r="AG2" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH2" s="2">
         <v>8</v>
       </c>
       <c r="AI2" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AJ2" s="3" t="s">
         <v>41</v>
@@ -824,7 +824,7 @@
         <v>39</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O3" s="4" t="s">
         <v>38</v>
@@ -881,13 +881,13 @@
         <v>38</v>
       </c>
       <c r="AG3" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AH3" s="4">
         <v>3</v>
       </c>
       <c r="AI3" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AJ3" s="5" t="s">
         <v>44</v>

</xml_diff>